<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@3e6519fd892acbb984c3eb7cfe0fc173bcc347da 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Medicatiegegevens.xlsx
+++ b/StructureDefinition-Medicatiegegevens.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-03T08:47:24+00:00</t>
+    <t>2025-03-04T09:51:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Medicatiegegevens abstract samenstelling voor het documenteren van de combinatie van Medicatieafspraak en Medicatiegebruik</t>
+    <t>Medicatiegegevens abstract samenstelling voor het documenteren van de combinatie van Medicatieafspraak en Medicatie Gebruik</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>